<commit_message>
Atualiza modelo de importação ICMS e normaliza permissão do .gitignore privado.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/planilhas/icms_importacao_modelo.xlsx
+++ b/planilhas/icms_importacao_modelo.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="59">
   <si>
     <t xml:space="preserve">id_cigam</t>
   </si>
@@ -197,12 +197,6 @@
   </si>
   <si>
     <t xml:space="preserve">001432</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PCT</t>
   </si>
 </sst>
 </file>
@@ -297,7 +291,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2148,1546 +2142,50 @@
         <v>14</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C46" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E46" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G46" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I46" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J46" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K46" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C47" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E47" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G47" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I47" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K47" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K48" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C49" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E49" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F49" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G49" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I49" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J49" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K49" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C50" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E50" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F50" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G50" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I50" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J50" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K50" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C51" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E51" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G51" s="1" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="H51" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I51" s="1" t="n">
-        <v>12</v>
-      </c>
-      <c r="J51" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K51" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C52" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E52" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F52" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G52" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H52" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I52" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J52" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K52" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C53" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E53" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G53" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H53" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I53" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K53" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C54" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E54" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G54" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I54" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K54" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C55" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E55" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G55" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I55" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K55" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C56" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E56" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G56" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I56" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K56" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C57" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E57" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G57" s="1" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="H57" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I57" s="1" t="n">
-        <v>12</v>
-      </c>
-      <c r="J57" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K57" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C58" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E58" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G58" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I58" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K58" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C59" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E59" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G59" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H59" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I59" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J59" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K59" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C60" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E60" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G60" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H60" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I60" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J60" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K60" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C61" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E61" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F61" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G61" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H61" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I61" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J61" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K61" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C62" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E62" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G62" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H62" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I62" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J62" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K62" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C63" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E63" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G63" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H63" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I63" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J63" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K63" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C64" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E64" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F64" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G64" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H64" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I64" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J64" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K64" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C65" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E65" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G65" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H65" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I65" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K65" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C66" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E66" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F66" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G66" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I66" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J66" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K66" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C67" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E67" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F67" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G67" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I67" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J67" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C68" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D68" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E68" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F68" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G68" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H68" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I68" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J68" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K68" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C69" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E69" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F69" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G69" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H69" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I69" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J69" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K69" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C70" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D70" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E70" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F70" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G70" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H70" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I70" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J70" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C71" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D71" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E71" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G71" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H71" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I71" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J71" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K71" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C72" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E72" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G72" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H72" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I72" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J72" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K72" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C73" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E73" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G73" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H73" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I73" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J73" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K73" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C74" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D74" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E74" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F74" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G74" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H74" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I74" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J74" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K74" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C75" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E75" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F75" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G75" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H75" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I75" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J75" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K75" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C76" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D76" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E76" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F76" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G76" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H76" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I76" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J76" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K76" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C77" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D77" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E77" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F77" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G77" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H77" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I77" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J77" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K77" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C78" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D78" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E78" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F78" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G78" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H78" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I78" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J78" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K78" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C79" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D79" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E79" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G79" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H79" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I79" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J79" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K79" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C80" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D80" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E80" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F80" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G80" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H80" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I80" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J80" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K80" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C81" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D81" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E81" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G81" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H81" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I81" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J81" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K81" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C82" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D82" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E82" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F82" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G82" s="1" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="H82" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I82" s="1" t="n">
-        <v>12</v>
-      </c>
-      <c r="J82" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K82" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C83" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D83" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E83" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F83" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G83" s="1" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="H83" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I83" s="1" t="n">
-        <v>12</v>
-      </c>
-      <c r="J83" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K83" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C84" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D84" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E84" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F84" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G84" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H84" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I84" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J84" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K84" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B85" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C85" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D85" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E85" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F85" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G85" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H85" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I85" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J85" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K85" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C86" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D86" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E86" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F86" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G86" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H86" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I86" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J86" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K86" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C87" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D87" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E87" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F87" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G87" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H87" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I87" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J87" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K87" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C88" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D88" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E88" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F88" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G88" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H88" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I88" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J88" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K88" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B89" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C89" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D89" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E89" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F89" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G89" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H89" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I89" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J89" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K89" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>